<commit_message>
Added support for mknotebooks with custom css
</commit_message>
<xml_diff>
--- a/src/Assets/Tables.xlsx
+++ b/src/Assets/Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/ELEMEMTS_H/company/github/harsh-maheshwari.github.io/src/Assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119969AD-D3CD-2D4C-BF2C-33A97DA2F978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{151B67D5-AC37-C74E-94B3-568551698C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{34CD1E43-5044-FC47-9ADD-5FB11EB3BB61}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20200" xr2:uid="{34CD1E43-5044-FC47-9ADD-5FB11EB3BB61}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="247">
   <si>
     <t>False positive (FP), type I error, false alarm, overestimation</t>
   </si>
@@ -496,35 +496,293 @@
     <t>Batch scoring: N/A —aggregates like these are computed      based on real-time events. Online prediction: Not Possible .</t>
   </si>
   <si>
-    <t>[Data Analytics Services for MSMEs](Services/2022-12-29 Services#data-analytics-services-for-msmes)</t>
-  </si>
-  <si>
-    <t>[Predictive Data Modeling and Forecasting](Services/2022-12-29 Services#predictive-data-modeling-and-forecasting)</t>
-  </si>
-  <si>
-    <t>[Data Science Consulting Services](Services/2022-12-29 Services#data-science-consulting-services)</t>
-  </si>
-  <si>
-    <t>[Data Integration Software Development](Services/2022-12-29 Services#data-integration-software-development)</t>
-  </si>
-  <si>
-    <t>[Data Science Recruitment](Services/2022-12-29 Services#data-science-recruitment)</t>
-  </si>
-  <si>
-    <t>[Data Science Education and Training](Services/2022-12-29 Services#data-science-education-and-training)</t>
-  </si>
-  <si>
-    <t>[Product and Market Development](Services/2022-12-29 Services#product-and-market-development)</t>
-  </si>
-  <si>
-    <t>Services</t>
+    <t>Concept</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Risk factor calculation</t>
+  </si>
+  <si>
+    <t>Size: Market equity (ME)</t>
+  </si>
+  <si>
+    <t>SMB</t>
+  </si>
+  <si>
+    <t>Small minus big</t>
+  </si>
+  <si>
+    <t>Nine small stock PF minus nine large stock PF.</t>
+  </si>
+  <si>
+    <t>Value: Book value of equity (BE) divided by ME</t>
+  </si>
+  <si>
+    <t>HML</t>
+  </si>
+  <si>
+    <t>High minus low</t>
+  </si>
+  <si>
+    <t>Two value PF minus two growth (with low BE/ME value) PF.</t>
+  </si>
+  <si>
+    <t>Operating profitability (OP): Revenue minus cost of goods sold/assets</t>
+  </si>
+  <si>
+    <t>RMW</t>
+  </si>
+  <si>
+    <t>Robust minus weak</t>
+  </si>
+  <si>
+    <t>Two robust OP PF minus two weak OP PF.</t>
+  </si>
+  <si>
+    <t>Investment: Investment/assets</t>
+  </si>
+  <si>
+    <t>CMA</t>
+  </si>
+  <si>
+    <t>Conservative minus aggressive</t>
+  </si>
+  <si>
+    <t>Two conservative investment portfolios, minus two aggressive investment portfolios.</t>
+  </si>
+  <si>
+    <t>Market</t>
+  </si>
+  <si>
+    <t>Rm-Rf</t>
+  </si>
+  <si>
+    <t>Excess return on the market</t>
+  </si>
+  <si>
+    <t>Value-weight return of all firms incorporated in and listed on major US exchanges with good data, minus the one-month Treasury bill rate.</t>
+  </si>
+  <si>
+    <t>Instrument</t>
+  </si>
+  <si>
+    <t>Buy Order [BO]</t>
+  </si>
+  <si>
+    <t>Sell Order [SO]</t>
+  </si>
+  <si>
+    <t>Calculation</t>
+  </si>
+  <si>
+    <t>Gold</t>
+  </si>
+  <si>
+    <t>Entry</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>FSL</t>
+  </si>
+  <si>
+    <t>MSL</t>
+  </si>
+  <si>
+    <t>TSL</t>
+  </si>
+  <si>
+    <t>Buy / Long</t>
+  </si>
+  <si>
+    <t>3DHH + 0.12%</t>
+  </si>
+  <si>
+    <t>Buy Entry + 1.2%</t>
+  </si>
+  <si>
+    <t>Max (MSL,TSL)</t>
+  </si>
+  <si>
+    <t>Buy Entry -1.2%</t>
+  </si>
+  <si>
+    <t>2DLL - 0.12%</t>
+  </si>
+  <si>
+    <t>Sell / Short</t>
+  </si>
+  <si>
+    <t>3DLL - 0.12%</t>
+  </si>
+  <si>
+    <t>Sell Entry - 1.2%</t>
+  </si>
+  <si>
+    <t>Min (MSL,TSL)</t>
+  </si>
+  <si>
+    <t>Sell Entry +1.2%</t>
+  </si>
+  <si>
+    <t>2DHH + 0.12%</t>
+  </si>
+  <si>
+    <t>Silver</t>
+  </si>
+  <si>
+    <t>2DHH + 0.2%</t>
+  </si>
+  <si>
+    <t>Buy Entry + 2%</t>
+  </si>
+  <si>
+    <t>Buy Entry - 2%</t>
+  </si>
+  <si>
+    <t>2DLL - 0.2%</t>
+  </si>
+  <si>
+    <t>Sell Entry - 2%</t>
+  </si>
+  <si>
+    <t>Sell Entry + 2%</t>
+  </si>
+  <si>
+    <t>Crude</t>
+  </si>
+  <si>
+    <t>2DHH + 0.4%</t>
+  </si>
+  <si>
+    <t>Buy Entry + 4%</t>
+  </si>
+  <si>
+    <t>Buy Entry - 4%</t>
+  </si>
+  <si>
+    <t>2DLL - 0.4%</t>
+  </si>
+  <si>
+    <t>Sell Entry - 4%</t>
+  </si>
+  <si>
+    <t>Sell Entry + 4%</t>
+  </si>
+  <si>
+    <t>Bank Nifty Futures</t>
+  </si>
+  <si>
+    <t>2DHH + 0.15%</t>
+  </si>
+  <si>
+    <t>Buy Entry + 1.5%</t>
+  </si>
+  <si>
+    <t>Buy Entry - 1.5%</t>
+  </si>
+  <si>
+    <t>2DLL - 0.15%</t>
+  </si>
+  <si>
+    <t>Sell Entry - 1.5%</t>
+  </si>
+  <si>
+    <t>Sell Entry + 1.5%</t>
+  </si>
+  <si>
+    <t>Nifty Futures</t>
+  </si>
+  <si>
+    <t>Buy Entry - 1.2%</t>
+  </si>
+  <si>
+    <t>Sell Entry + 1.2%</t>
+  </si>
+  <si>
+    <t>Stock Futures</t>
+  </si>
+  <si>
+    <t>BO / SO</t>
+  </si>
+  <si>
+    <t>Lots</t>
+  </si>
+  <si>
+    <t>Trigger Price / Price</t>
+  </si>
+  <si>
+    <t>Nil</t>
+  </si>
+  <si>
+    <t>Buy and Target not achieved</t>
+  </si>
+  <si>
+    <t>Buy and Target achieved</t>
+  </si>
+  <si>
+    <t>Sell and Target not achieved</t>
+  </si>
+  <si>
+    <t>Sell and Target achieved</t>
+  </si>
+  <si>
+    <t>Buy Entry</t>
+  </si>
+  <si>
+    <t>BO</t>
+  </si>
+  <si>
+    <t>Trigger Price</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Buy Target</t>
+  </si>
+  <si>
+    <t>SO</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Buy Stop Loss 1</t>
+  </si>
+  <si>
+    <t>Buy Stop Loss 2</t>
+  </si>
+  <si>
+    <t>Sell Entry</t>
+  </si>
+  <si>
+    <t>Sell Target</t>
+  </si>
+  <si>
+    <t>Sell Stop Loss 1</t>
+  </si>
+  <si>
+    <t>Sell Stop Loss 2</t>
+  </si>
+  <si>
+    <t>Position Entries</t>
+  </si>
+  <si>
+    <t>Trade Step</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -540,16 +798,77 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Montserrat"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Montserrat"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Montserrat"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Montserrat"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA4C2F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB6D7A8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA9999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE599"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -557,11 +876,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -572,7 +943,70 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -889,7 +1323,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{095F115B-440C-0845-90BD-CDCAD3191863}">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="44.1640625" style="1" customWidth="1"/>
@@ -902,13 +1336,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -1068,38 +1502,926 @@
         <v>29</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A51" s="1" t="s">
+    <row r="58" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D60" s="7" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A52" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A53" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A55" s="1" t="s">
-        <v>159</v>
+    <row r="61" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B74" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="C74" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="E74" s="13"/>
+      <c r="F74" s="13"/>
+    </row>
+    <row r="75" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B75" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C75" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D75" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E75" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="F75" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B76" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="C76" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="D76" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="E76" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="F76" s="19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="C77" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="D77" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="E77" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="F77" s="19" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B78" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D78" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E78" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="F78" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B79" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="C79" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="D79" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="E79" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="F79" s="19" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B80" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="C80" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="D80" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="E80" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="F80" s="19" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="B81" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C81" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D81" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E81" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="F81" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B82" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="C82" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="D82" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="E82" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="F82" s="19" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B83" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="C83" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="D83" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="E83" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="F83" s="19" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="B84" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C84" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D84" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E84" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="F84" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B85" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="C85" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="D85" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="E85" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="F85" s="19" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B86" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="C86" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="D86" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="E86" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="F86" s="19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B87" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C87" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D87" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E87" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="F87" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B88" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="C88" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="D88" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="E88" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="F88" s="19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B89" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C89" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="D89" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="E89" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="F89" s="19" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B90" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C90" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D90" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E90" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="F90" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B91" s="20"/>
+      <c r="C91" s="21"/>
+      <c r="D91" s="21"/>
+      <c r="E91" s="22"/>
+      <c r="F91" s="22"/>
+    </row>
+    <row r="92" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B92" s="21"/>
+      <c r="C92" s="20"/>
+      <c r="D92" s="20"/>
+      <c r="E92" s="22"/>
+      <c r="F92" s="22"/>
+    </row>
+    <row r="94" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:9" ht="37" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="24" t="s">
+        <v>245</v>
+      </c>
+      <c r="B95" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="C95" s="23" t="s">
+        <v>225</v>
+      </c>
+      <c r="D95" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="E95" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="F95" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="G95" s="23" t="s">
+        <v>229</v>
+      </c>
+      <c r="H95" s="23" t="s">
+        <v>230</v>
+      </c>
+      <c r="I95" s="23" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="24" t="s">
+        <v>232</v>
+      </c>
+      <c r="B96" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="C96" s="25">
+        <v>2</v>
+      </c>
+      <c r="D96" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="E96" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="F96" s="25"/>
+      <c r="G96" s="25"/>
+      <c r="H96" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="I96" s="25" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="24" t="s">
+        <v>236</v>
+      </c>
+      <c r="B97" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="C97" s="25">
+        <v>1</v>
+      </c>
+      <c r="D97" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="E97" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="F97" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="G97" s="25"/>
+      <c r="H97" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="I97" s="25" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="24" t="s">
+        <v>239</v>
+      </c>
+      <c r="B98" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="C98" s="25">
+        <v>2</v>
+      </c>
+      <c r="D98" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="E98" s="25"/>
+      <c r="F98" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="G98" s="25"/>
+      <c r="H98" s="25"/>
+      <c r="I98" s="25"/>
+    </row>
+    <row r="99" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="B99" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="C99" s="25">
+        <v>1</v>
+      </c>
+      <c r="D99" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="E99" s="25"/>
+      <c r="F99" s="25"/>
+      <c r="G99" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="H99" s="25"/>
+      <c r="I99" s="25"/>
+    </row>
+    <row r="100" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="24" t="s">
+        <v>241</v>
+      </c>
+      <c r="B100" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="C100" s="25">
+        <v>2</v>
+      </c>
+      <c r="D100" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="E100" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="F100" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="G100" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="H100" s="25"/>
+      <c r="I100" s="25"/>
+    </row>
+    <row r="101" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="B101" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="C101" s="25">
+        <v>1</v>
+      </c>
+      <c r="D101" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="E101" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="F101" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="G101" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="H101" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="I101" s="25"/>
+    </row>
+    <row r="102" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="24" t="s">
+        <v>243</v>
+      </c>
+      <c r="B102" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="C102" s="25">
+        <v>2</v>
+      </c>
+      <c r="D102" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="E102" s="25"/>
+      <c r="F102" s="25"/>
+      <c r="G102" s="25"/>
+      <c r="H102" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="I102" s="25"/>
+    </row>
+    <row r="103" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="24" t="s">
+        <v>244</v>
+      </c>
+      <c r="B103" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="C103" s="25">
+        <v>1</v>
+      </c>
+      <c r="D103" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="E103" s="25"/>
+      <c r="F103" s="25"/>
+      <c r="G103" s="25"/>
+      <c r="H103" s="25"/>
+      <c r="I103" s="25" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B106" s="9"/>
+      <c r="C106" s="10"/>
+      <c r="D106" s="11"/>
+      <c r="E106" s="12"/>
+      <c r="F106" s="13"/>
+      <c r="G106" s="13"/>
+    </row>
+    <row r="107" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B107" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="C107" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="D107" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="E107" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="F107" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="G107" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B108" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="C108" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="D108" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="E108" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F108" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="G108" s="19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B109" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="C109" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="D109" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="E109" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="F109" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="G109" s="19" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B110" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="C110" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="D110" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="E110" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F110" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="G110" s="19" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B111" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="C111" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="D111" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="E111" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="F111" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="G111" s="19" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="B112" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="C112" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="D112" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="E112" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F112" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="G112" s="19" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="B113" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="C113" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="D113" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="E113" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="F113" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="G113" s="19" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="B114" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="C114" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="D114" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="E114" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F114" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="G114" s="19" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="B115" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="C115" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="D115" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="E115" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="F115" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="G115" s="19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B116" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="C116" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="D116" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="E116" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F116" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="G116" s="19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B117" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="C117" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="D117" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="E117" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="F117" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="G117" s="19" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>